<commit_message>
add git workflow (branch off dev, feature branch per task) to delegation
</commit_message>
<xml_diff>
--- a/Group11_Delegation_Timeline.xlsx
+++ b/Group11_Delegation_Timeline.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Check-ins" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="API Contract" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Git workflow" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Timeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tasks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Check-ins" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="API Contract" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$4:$H$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tasks'!$A$4:$H$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="ddd mmm d"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,6 +96,22 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001D1D1F"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001D1D1F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="00047857"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
       <color rgb="001D1D1F"/>
       <sz val="10"/>
     </font>
@@ -199,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -249,22 +266,37 @@
     <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,7 +305,7 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -285,7 +317,7 @@
     <xf numFmtId="0" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -318,7 +350,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -968,6 +1000,260 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Git workflow — everyone follows this</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Always branch off dev. Never commit straight to main or dev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Before you start ANY task — always:</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>git checkout dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>git pull origin dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>git checkout -b &lt;branch&gt;   # branch off the latest dev</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Release / defense-ready</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Updated only at Saturday gates, after QA sign-off. Never commit directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>dev</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Integration branch</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Everything merges here first via Pull Request. Never commit directly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>feature branch</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>One per task</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Branched off the latest dev; deleted after it merges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Branch prefix</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Examples</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Front end</t>
+        </is>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>fe/</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>fe/route-query, fe/compare-view</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Backend / algorithm</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>be/</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>be/astar-core, be/compare-endpoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>ml/</t>
+        </is>
+      </c>
+      <c r="C17" s="21" t="inlineStr">
+        <is>
+          <t>ml/ahp-weights, ml/lstm-ridership</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>QA / tests</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>qa/</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>qa/comparison-check</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>• Commit small and often; lowercase messages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>• Push your branch: git push -u origin &lt;branch&gt;.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>• Open a Pull Request into dev. Dave (QA) reviews &amp; signs off BEFORE it merges into dev.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>• Release: dev -&gt; main only at the Saturday check-in gates, once QA has signed off.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1019,46 +1305,46 @@
           <t>Kickoff</t>
         </is>
       </c>
-      <c r="B5" s="17" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>Mon Jul 13</t>
         </is>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Align on API contract; assign; Figma finalized from mockup v4.</t>
         </is>
       </c>
-      <c r="D5" s="17" t="inlineStr">
+      <c r="D5" s="23" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="6" ht="74" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Week 1</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>Jul 13 – Jul 18</t>
         </is>
       </c>
-      <c r="C6" s="19" t="inlineStr">
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>FRONT END BUILD. Luis: all 4 screens in Bootstrap 5 + design system + copy fixes. Andrei: lock API contract, Express skeleton, graph static attrs. Princess: start AHP matrices. Dave: test plan.</t>
         </is>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>Sat Jul 18 — ★ UI/UX dashboard COMPLETE; API contract locked &amp; documented.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="74" customHeight="1">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>Week 2</t>
         </is>
@@ -1080,29 +1366,29 @@
       </c>
     </row>
     <row r="8" ht="74" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
         <is>
           <t>Week 3</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Jul 27 – Aug 1</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>ML + BENCHMARK. LSTM (ridership) + RFR (flood) integrated; dynamic edges refresh; benchmark harness → 360 rows. Luis: polish comparison view. Dave: comparison check.</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>Sat Aug 1 — 360-row benchmark with 8 KPIs; routes differ across profiles.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="74" customHeight="1">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>Week 4</t>
         </is>
@@ -1129,17 +1415,17 @@
           <t>Buffer</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="23" t="inlineStr">
         <is>
           <t>Aug 10 – Aug 15</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>Defense prep, last fixes, rehearsal, dry runs. No new features.</t>
         </is>
       </c>
-      <c r="D10" s="17" t="inlineStr">
+      <c r="D10" s="23" t="inlineStr">
         <is>
           <t>Sat Aug 15 — ★ Prototype complete &amp; defense-ready (hard deadline).</t>
         </is>
@@ -1154,7 +1440,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1238,7 +1524,7 @@
           <t>Kickoff meeting + assign + align on API contract</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="26" t="inlineStr">
         <is>
           <t>All</t>
         </is>
@@ -1248,15 +1534,15 @@
           <t>Planning</t>
         </is>
       </c>
-      <c r="E5" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F5" s="23" t="n">
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="n">
         <v>46216</v>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="28" t="n">
         <v>46216</v>
       </c>
       <c r="H5" s="8" t="inlineStr">
@@ -1274,7 +1560,7 @@
           <t>Finalize Figma from mockup v4</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1284,15 +1570,15 @@
           <t>Design</t>
         </is>
       </c>
-      <c r="E6" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F6" s="23" t="n">
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="n">
         <v>46216</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="28" t="n">
         <v>46218</v>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -1310,7 +1596,7 @@
           <t>Agree API request/response shape with Andrei</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1320,15 +1606,15 @@
           <t>Handoff</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F7" s="23" t="n">
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="n">
         <v>46217</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="28" t="n">
         <v>46218</v>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -1346,7 +1632,7 @@
           <t>Network map render: 10 anchors, 3 rail lines, legend, stat chips</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C8" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1356,15 +1642,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="n">
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="n">
         <v>46218</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="28" t="n">
         <v>46219</v>
       </c>
       <c r="H8" s="8" t="inlineStr">
@@ -1382,7 +1668,7 @@
           <t>Route query screen: OD dropdowns, profile selector, validation, loading</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1392,15 +1678,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F9" s="23" t="n">
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="n">
         <v>46219</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="28" t="n">
         <v>46220</v>
       </c>
       <c r="H9" s="8" t="inlineStr">
@@ -1418,7 +1704,7 @@
           <t>Result view: map, why-this-route, criteria rings, 4 headline stats</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1428,15 +1714,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F10" s="23" t="n">
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="n">
         <v>46220</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H10" s="8" t="inlineStr">
@@ -1454,7 +1740,7 @@
           <t>Comparison view: 4 cards, active highlight, transparency frame + cost eq (money shot)</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1464,15 +1750,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F11" s="23" t="n">
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="n">
         <v>46220</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H11" s="8" t="inlineStr">
@@ -1490,7 +1776,7 @@
           <t>Design system: color tokens, all states (default/hover/active/disabled/loading/empty/error), responsive</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1500,15 +1786,15 @@
           <t>Design</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F12" s="23" t="n">
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="n">
         <v>46218</v>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G12" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H12" s="8" t="inlineStr">
@@ -1526,7 +1812,7 @@
           <t>Copy fixes: drop 'reimagined' &amp; 'live PAGASA' -&gt; 'PAGASA TenDay Forecast', framework voice</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1536,15 +1822,15 @@
           <t>Copy</t>
         </is>
       </c>
-      <c r="E13" s="25" t="inlineStr">
+      <c r="E13" s="30" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F13" s="23" t="n">
+      <c r="F13" s="28" t="n">
         <v>46221</v>
       </c>
-      <c r="G13" s="23" t="n">
+      <c r="G13" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
@@ -1554,36 +1840,36 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="26" t="n">
+      <c r="A14" s="31" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>★ MILESTONE: UI/UX dashboard COMPLETE</t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
       </c>
-      <c r="D14" s="26" t="inlineStr">
+      <c r="D14" s="31" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="E14" s="29" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F14" s="30" t="n">
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F14" s="35" t="n">
         <v>46221</v>
       </c>
-      <c r="G14" s="30" t="n">
+      <c r="G14" s="35" t="n">
         <v>46221</v>
       </c>
-      <c r="H14" s="26" t="inlineStr">
+      <c r="H14" s="31" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
@@ -1598,7 +1884,7 @@
           <t>Wire front end to live /route + /compare</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1608,15 +1894,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F15" s="23" t="n">
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F15" s="28" t="n">
         <v>46223</v>
       </c>
-      <c r="G15" s="23" t="n">
+      <c r="G15" s="28" t="n">
         <v>46228</v>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -1634,7 +1920,7 @@
           <t>Polish comparison view for panel</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1644,15 +1930,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F16" s="23" t="n">
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="n">
         <v>46230</v>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="28" t="n">
         <v>46235</v>
       </c>
       <c r="H16" s="8" t="inlineStr">
@@ -1670,7 +1956,7 @@
           <t>Responsive QA fixes with Dave</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="29" t="inlineStr">
         <is>
           <t>Luis</t>
         </is>
@@ -1680,15 +1966,15 @@
           <t>Front end</t>
         </is>
       </c>
-      <c r="E17" s="25" t="inlineStr">
+      <c r="E17" s="30" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F17" s="23" t="n">
+      <c r="F17" s="28" t="n">
         <v>46237</v>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="28" t="n">
         <v>46242</v>
       </c>
       <c r="H17" s="8" t="inlineStr">
@@ -1706,7 +1992,7 @@
           <t>Finalize + document API contract (/route, /compare)</t>
         </is>
       </c>
-      <c r="C18" s="31" t="inlineStr">
+      <c r="C18" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1716,15 +2002,15 @@
           <t>API</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="n">
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F18" s="28" t="n">
         <v>46216</v>
       </c>
-      <c r="G18" s="23" t="n">
+      <c r="G18" s="28" t="n">
         <v>46218</v>
       </c>
       <c r="H18" s="8" t="inlineStr">
@@ -1742,7 +2028,7 @@
           <t>Express routing service skeleton</t>
         </is>
       </c>
-      <c r="C19" s="31" t="inlineStr">
+      <c r="C19" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1752,15 +2038,15 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F19" s="23" t="n">
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="n">
         <v>46218</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="28" t="n">
         <v>46220</v>
       </c>
       <c r="H19" s="8" t="inlineStr">
@@ -1778,7 +2064,7 @@
           <t>Graph layer: load static attrs at startup (fare, base time, distance, transfer flags)</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1788,15 +2074,15 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E20" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="n">
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="n">
         <v>46219</v>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H20" s="8" t="inlineStr">
@@ -1814,7 +2100,7 @@
           <t>Multi-criteria A*: Eq 3 cost, heuristic v_max 60, mode speeds 40/60/30/20, multiplier 1.0-2.0</t>
         </is>
       </c>
-      <c r="C21" s="31" t="inlineStr">
+      <c r="C21" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1824,15 +2110,15 @@
           <t>Algorithm</t>
         </is>
       </c>
-      <c r="E21" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F21" s="23" t="n">
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F21" s="28" t="n">
         <v>46223</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="28" t="n">
         <v>46225</v>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -1850,7 +2136,7 @@
           <t>Node-expansion counter inside the loop (pruning evidence)</t>
         </is>
       </c>
-      <c r="C22" s="31" t="inlineStr">
+      <c r="C22" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1860,15 +2146,15 @@
           <t>Algorithm</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F22" s="23" t="n">
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F22" s="28" t="n">
         <v>46225</v>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="28" t="n">
         <v>46226</v>
       </c>
       <c r="H22" s="8" t="inlineStr">
@@ -1886,7 +2172,7 @@
           <t>Distance-based A* baseline (locked comparison target)</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1896,15 +2182,15 @@
           <t>Algorithm</t>
         </is>
       </c>
-      <c r="E23" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F23" s="23" t="n">
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F23" s="28" t="n">
         <v>46226</v>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="28" t="n">
         <v>46227</v>
       </c>
       <c r="H23" s="8" t="inlineStr">
@@ -1922,7 +2208,7 @@
           <t>Transfer friction TF-prime from 5x5 adjacency matrix</t>
         </is>
       </c>
-      <c r="C24" s="31" t="inlineStr">
+      <c r="C24" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1932,15 +2218,15 @@
           <t>Algorithm</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F24" s="23" t="n">
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F24" s="28" t="n">
         <v>46226</v>
       </c>
-      <c r="G24" s="23" t="n">
+      <c r="G24" s="28" t="n">
         <v>46227</v>
       </c>
       <c r="H24" s="8" t="inlineStr">
@@ -1958,7 +2244,7 @@
           <t>POST /route: one route + 8 KPIs</t>
         </is>
       </c>
-      <c r="C25" s="31" t="inlineStr">
+      <c r="C25" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -1968,15 +2254,15 @@
           <t>API</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F25" s="23" t="n">
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="n">
         <v>46227</v>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G25" s="28" t="n">
         <v>46228</v>
       </c>
       <c r="H25" s="8" t="inlineStr">
@@ -1994,7 +2280,7 @@
           <t>POST /compare: 4 profiles + baseline = 5 results</t>
         </is>
       </c>
-      <c r="C26" s="31" t="inlineStr">
+      <c r="C26" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2004,15 +2290,15 @@
           <t>API</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F26" s="23" t="n">
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F26" s="28" t="n">
         <v>46227</v>
       </c>
-      <c r="G26" s="23" t="n">
+      <c r="G26" s="28" t="n">
         <v>46228</v>
       </c>
       <c r="H26" s="8" t="inlineStr">
@@ -2030,7 +2316,7 @@
           <t>LSTM ridership model (TF + Keras, 24-mo window, eFOI contingency)</t>
         </is>
       </c>
-      <c r="C27" s="31" t="inlineStr">
+      <c r="C27" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2040,15 +2326,15 @@
           <t>ML</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F27" s="23" t="n">
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F27" s="28" t="n">
         <v>46223</v>
       </c>
-      <c r="G27" s="23" t="n">
+      <c r="G27" s="28" t="n">
         <v>46232</v>
       </c>
       <c r="H27" s="8" t="inlineStr">
@@ -2066,7 +2352,7 @@
           <t>RFR flood-risk model (scikit-learn, PAGASA TenDay Forecast input)</t>
         </is>
       </c>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="C28" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2076,15 +2362,15 @@
           <t>ML</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F28" s="23" t="n">
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="n">
         <v>46225</v>
       </c>
-      <c r="G28" s="23" t="n">
+      <c r="G28" s="28" t="n">
         <v>46232</v>
       </c>
       <c r="H28" s="8" t="inlineStr">
@@ -2102,7 +2388,7 @@
           <t>Refresh dynamic edges (ridership, flood) at start of each benchmark run</t>
         </is>
       </c>
-      <c r="C29" s="31" t="inlineStr">
+      <c r="C29" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2112,15 +2398,15 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F29" s="23" t="n">
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F29" s="28" t="n">
         <v>46232</v>
       </c>
-      <c r="G29" s="23" t="n">
+      <c r="G29" s="28" t="n">
         <v>46233</v>
       </c>
       <c r="H29" s="8" t="inlineStr">
@@ -2138,7 +2424,7 @@
           <t>Benchmark harness: 45 OD x 4 profiles x 2 algos = 360 rows, 8 KPIs</t>
         </is>
       </c>
-      <c r="C30" s="31" t="inlineStr">
+      <c r="C30" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2148,15 +2434,15 @@
           <t>Benchmark</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F30" s="23" t="n">
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="n">
         <v>46233</v>
       </c>
-      <c r="G30" s="23" t="n">
+      <c r="G30" s="28" t="n">
         <v>46235</v>
       </c>
       <c r="H30" s="8" t="inlineStr">
@@ -2174,7 +2460,7 @@
           <t>Integration + fixes from QA</t>
         </is>
       </c>
-      <c r="C31" s="31" t="inlineStr">
+      <c r="C31" s="36" t="inlineStr">
         <is>
           <t>Andrei</t>
         </is>
@@ -2184,15 +2470,15 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F31" s="23" t="n">
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F31" s="28" t="n">
         <v>46237</v>
       </c>
-      <c r="G31" s="23" t="n">
+      <c r="G31" s="28" t="n">
         <v>46242</v>
       </c>
       <c r="H31" s="8" t="inlineStr">
@@ -2210,7 +2496,7 @@
           <t>AHP weight derivation (Excel): 150 respondents, Saaty 1-9, normalized col avg, reject CR&gt;=0.10</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C32" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2220,15 +2506,15 @@
           <t>ML</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F32" s="23" t="n">
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F32" s="28" t="n">
         <v>46216</v>
       </c>
-      <c r="G32" s="23" t="n">
+      <c r="G32" s="28" t="n">
         <v>46223</v>
       </c>
       <c r="H32" s="8" t="inlineStr">
@@ -2246,7 +2532,7 @@
           <t>Hand 4 AHP weight vectors to Andrei</t>
         </is>
       </c>
-      <c r="C33" s="32" t="inlineStr">
+      <c r="C33" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2256,15 +2542,15 @@
           <t>Handoff</t>
         </is>
       </c>
-      <c r="E33" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F33" s="23" t="n">
+      <c r="E33" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F33" s="28" t="n">
         <v>46223</v>
       </c>
-      <c r="G33" s="23" t="n">
+      <c r="G33" s="28" t="n">
         <v>46223</v>
       </c>
       <c r="H33" s="8" t="inlineStr">
@@ -2282,7 +2568,7 @@
           <t>Graph layer support: static attrs + dynamic edge refresh</t>
         </is>
       </c>
-      <c r="C34" s="32" t="inlineStr">
+      <c r="C34" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2292,15 +2578,15 @@
           <t>Backend</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F34" s="23" t="n">
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F34" s="28" t="n">
         <v>46219</v>
       </c>
-      <c r="G34" s="23" t="n">
+      <c r="G34" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H34" s="8" t="inlineStr">
@@ -2318,7 +2604,7 @@
           <t>Transfer friction: 5x5 adjacency matrix values</t>
         </is>
       </c>
-      <c r="C35" s="32" t="inlineStr">
+      <c r="C35" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2328,15 +2614,15 @@
           <t>ML</t>
         </is>
       </c>
-      <c r="E35" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F35" s="23" t="n">
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F35" s="28" t="n">
         <v>46218</v>
       </c>
-      <c r="G35" s="23" t="n">
+      <c r="G35" s="28" t="n">
         <v>46223</v>
       </c>
       <c r="H35" s="8" t="inlineStr">
@@ -2354,7 +2640,7 @@
           <t>LSTM/RFR support + training-data prep</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C36" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2364,15 +2650,15 @@
           <t>ML</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F36" s="23" t="n">
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F36" s="28" t="n">
         <v>46225</v>
       </c>
-      <c r="G36" s="23" t="n">
+      <c r="G36" s="28" t="n">
         <v>46232</v>
       </c>
       <c r="H36" s="8" t="inlineStr">
@@ -2390,7 +2676,7 @@
           <t>Documentation: methodology, model cards, data sources</t>
         </is>
       </c>
-      <c r="C37" s="32" t="inlineStr">
+      <c r="C37" s="37" t="inlineStr">
         <is>
           <t>Princess</t>
         </is>
@@ -2400,15 +2686,15 @@
           <t>Docs</t>
         </is>
       </c>
-      <c r="E37" s="25" t="inlineStr">
+      <c r="E37" s="30" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="F37" s="23" t="n">
+      <c r="F37" s="28" t="n">
         <v>46230</v>
       </c>
-      <c r="G37" s="23" t="n">
+      <c r="G37" s="28" t="n">
         <v>46242</v>
       </c>
       <c r="H37" s="8" t="inlineStr">
@@ -2426,7 +2712,7 @@
           <t>Draft test plan + test cases for all 4 screens</t>
         </is>
       </c>
-      <c r="C38" s="33" t="inlineStr">
+      <c r="C38" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2436,15 +2722,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F38" s="23" t="n">
+      <c r="E38" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F38" s="28" t="n">
         <v>46218</v>
       </c>
-      <c r="G38" s="23" t="n">
+      <c r="G38" s="28" t="n">
         <v>46221</v>
       </c>
       <c r="H38" s="8" t="inlineStr">
@@ -2462,7 +2748,7 @@
           <t>Functional QA of UI/UX dashboard</t>
         </is>
       </c>
-      <c r="C39" s="33" t="inlineStr">
+      <c r="C39" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2472,15 +2758,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F39" s="23" t="n">
+      <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F39" s="28" t="n">
         <v>46221</v>
       </c>
-      <c r="G39" s="23" t="n">
+      <c r="G39" s="28" t="n">
         <v>46223</v>
       </c>
       <c r="H39" s="8" t="inlineStr">
@@ -2498,7 +2784,7 @@
           <t>Set up test harness against API contract</t>
         </is>
       </c>
-      <c r="C40" s="33" t="inlineStr">
+      <c r="C40" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2508,15 +2794,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F40" s="23" t="n">
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F40" s="28" t="n">
         <v>46223</v>
       </c>
-      <c r="G40" s="23" t="n">
+      <c r="G40" s="28" t="n">
         <v>46228</v>
       </c>
       <c r="H40" s="8" t="inlineStr">
@@ -2534,7 +2820,7 @@
           <t>Functional QA: dropdowns=10 anchors, profiles=4, block same/empty OD, loading+error, geometry render</t>
         </is>
       </c>
-      <c r="C41" s="33" t="inlineStr">
+      <c r="C41" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2544,15 +2830,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F41" s="23" t="n">
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F41" s="28" t="n">
         <v>46230</v>
       </c>
-      <c r="G41" s="23" t="n">
+      <c r="G41" s="28" t="n">
         <v>46234</v>
       </c>
       <c r="H41" s="8" t="inlineStr">
@@ -2570,7 +2856,7 @@
           <t>Comparison check: 4 profiles give different routes; flag loud if any two match</t>
         </is>
       </c>
-      <c r="C42" s="33" t="inlineStr">
+      <c r="C42" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2580,15 +2866,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F42" s="23" t="n">
+      <c r="E42" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F42" s="28" t="n">
         <v>46234</v>
       </c>
-      <c r="G42" s="23" t="n">
+      <c r="G42" s="28" t="n">
         <v>46235</v>
       </c>
       <c r="H42" s="8" t="inlineStr">
@@ -2606,7 +2892,7 @@
           <t>Data pipeline: log = exactly 360 rows, 8 KPIs incl. fare with 20% student/senior discount</t>
         </is>
       </c>
-      <c r="C43" s="33" t="inlineStr">
+      <c r="C43" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2616,15 +2902,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F43" s="23" t="n">
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F43" s="28" t="n">
         <v>46237</v>
       </c>
-      <c r="G43" s="23" t="n">
+      <c r="G43" s="28" t="n">
         <v>46238</v>
       </c>
       <c r="H43" s="8" t="inlineStr">
@@ -2642,7 +2928,7 @@
           <t>Pruning check: framework nodes expanded &lt; baseline on pruned queries; flag if not</t>
         </is>
       </c>
-      <c r="C44" s="33" t="inlineStr">
+      <c r="C44" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2652,15 +2938,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F44" s="23" t="n">
+      <c r="E44" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F44" s="28" t="n">
         <v>46238</v>
       </c>
-      <c r="G44" s="23" t="n">
+      <c r="G44" s="28" t="n">
         <v>46239</v>
       </c>
       <c r="H44" s="8" t="inlineStr">
@@ -2678,7 +2964,7 @@
           <t>Final QA sign-off before merge</t>
         </is>
       </c>
-      <c r="C45" s="33" t="inlineStr">
+      <c r="C45" s="38" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
@@ -2688,15 +2974,15 @@
           <t>QA</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F45" s="23" t="n">
+      <c r="E45" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F45" s="28" t="n">
         <v>46240</v>
       </c>
-      <c r="G45" s="23" t="n">
+      <c r="G45" s="28" t="n">
         <v>46242</v>
       </c>
       <c r="H45" s="8" t="inlineStr">
@@ -2714,7 +3000,7 @@
           <t>Integration freeze + full dry run</t>
         </is>
       </c>
-      <c r="C46" s="21" t="inlineStr">
+      <c r="C46" s="26" t="inlineStr">
         <is>
           <t>All</t>
         </is>
@@ -2724,15 +3010,15 @@
           <t>Integration</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F46" s="23" t="n">
+      <c r="E46" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F46" s="28" t="n">
         <v>46242</v>
       </c>
-      <c r="G46" s="23" t="n">
+      <c r="G46" s="28" t="n">
         <v>46242</v>
       </c>
       <c r="H46" s="8" t="inlineStr">
@@ -2750,7 +3036,7 @@
           <t>Buffer / defense prep / rehearsal / dry runs</t>
         </is>
       </c>
-      <c r="C47" s="21" t="inlineStr">
+      <c r="C47" s="26" t="inlineStr">
         <is>
           <t>All</t>
         </is>
@@ -2760,15 +3046,15 @@
           <t>Buffer</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F47" s="23" t="n">
+      <c r="E47" s="27" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F47" s="28" t="n">
         <v>46244</v>
       </c>
-      <c r="G47" s="23" t="n">
+      <c r="G47" s="28" t="n">
         <v>46249</v>
       </c>
       <c r="H47" s="8" t="inlineStr">
@@ -2778,36 +3064,36 @@
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="26" t="n">
+      <c r="A48" s="31" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="27" t="inlineStr">
+      <c r="B48" s="32" t="inlineStr">
         <is>
           <t>★ MILESTONE: Prototype complete &amp; defense-ready (hard deadline)</t>
         </is>
       </c>
-      <c r="C48" s="34" t="inlineStr">
+      <c r="C48" s="39" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="D48" s="26" t="inlineStr">
+      <c r="D48" s="31" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="E48" s="29" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="F48" s="30" t="n">
+      <c r="E48" s="34" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F48" s="35" t="n">
         <v>46249</v>
       </c>
-      <c r="G48" s="30" t="n">
+      <c r="G48" s="35" t="n">
         <v>46249</v>
       </c>
-      <c r="H48" s="26" t="inlineStr">
+      <c r="H48" s="31" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
@@ -2823,7 +3109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2869,17 +3155,17 @@
       </c>
     </row>
     <row r="5" ht="84" customHeight="1">
-      <c r="A5" s="35" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>#1</t>
         </is>
       </c>
-      <c r="B5" s="36" t="inlineStr">
+      <c r="B5" s="41" t="inlineStr">
         <is>
           <t>Sat Jul 18</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>★ UI/UX dashboard COMPLETE — all 4 screens in Bootstrap 5 with all states.
 API contract locked &amp; documented (Andrei).
@@ -2889,7 +3175,7 @@
       </c>
     </row>
     <row r="6" ht="84" customHeight="1">
-      <c r="A6" s="37" t="inlineStr">
+      <c r="A6" s="42" t="inlineStr">
         <is>
           <t>#2</t>
         </is>
@@ -2909,17 +3195,17 @@
       </c>
     </row>
     <row r="7" ht="84" customHeight="1">
-      <c r="A7" s="35" t="inlineStr">
+      <c r="A7" s="40" t="inlineStr">
         <is>
           <t>#3</t>
         </is>
       </c>
-      <c r="B7" s="36" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>Sat Aug 1</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>LSTM + RFR integrated; dynamic edges refresh at run start.
 Benchmark harness produces exactly 360 rows with all 8 KPIs.
@@ -2929,7 +3215,7 @@
       </c>
     </row>
     <row r="8" ht="84" customHeight="1">
-      <c r="A8" s="37" t="inlineStr">
+      <c r="A8" s="42" t="inlineStr">
         <is>
           <t>#4</t>
         </is>
@@ -2949,17 +3235,17 @@
       </c>
     </row>
     <row r="9" ht="84" customHeight="1">
-      <c r="A9" s="38" t="inlineStr">
+      <c r="A9" s="43" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="B9" s="26" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>Sat Aug 15</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>★ Prototype complete &amp; defense-ready. Buffer week used only for defense prep, rehearsal, and last fixes — no new features.</t>
         </is>
@@ -2974,7 +3260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3014,7 +3300,7 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="39" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>POST /route</t>
         </is>
@@ -3026,7 +3312,7 @@
           <t>Request</t>
         </is>
       </c>
-      <c r="B6" s="40" t="inlineStr">
+      <c r="B6" s="45" t="inlineStr">
         <is>
           <t>{ origin: &lt;anchorId&gt;, destination: &lt;anchorId&gt;, profile: 'uncrowded'|'cheapest'|'safest'|'convenient' }</t>
         </is>
@@ -3050,7 +3336,7 @@
           <t>Response</t>
         </is>
       </c>
-      <c r="B8" s="40" t="inlineStr">
+      <c r="B8" s="45" t="inlineStr">
         <is>
           <t>{ profile, origin, destination, geometry: [[lat,lng], ...], kpis: {...}, why_this_route: &lt;text&gt;, criteria: { T, F, R, P } }</t>
         </is>
@@ -3069,7 +3355,7 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="39" t="inlineStr">
+      <c r="A10" s="44" t="inlineStr">
         <is>
           <t>POST /compare</t>
         </is>
@@ -3081,7 +3367,7 @@
           <t>Request</t>
         </is>
       </c>
-      <c r="B11" s="40" t="inlineStr">
+      <c r="B11" s="45" t="inlineStr">
         <is>
           <t>{ origin: &lt;anchorId&gt;, destination: &lt;anchorId&gt; }</t>
         </is>
@@ -3093,7 +3379,7 @@
           <t>Response</t>
         </is>
       </c>
-      <c r="B12" s="40" t="inlineStr">
+      <c r="B12" s="45" t="inlineStr">
         <is>
           <t>{ origin, destination, results: [ { profile: 'baseline'|&lt;4 profiles&gt;, geometry, kpis } ] }  -&gt; 5 results (4 profiles + distance baseline)</t>
         </is>
@@ -3112,7 +3398,7 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="44" t="inlineStr">
         <is>
           <t>Benchmark log</t>
         </is>
@@ -3136,7 +3422,7 @@
           <t>Columns</t>
         </is>
       </c>
-      <c r="B16" s="40" t="inlineStr">
+      <c r="B16" s="45" t="inlineStr">
         <is>
           <t>od_pair, profile, algorithm, then the 8 KPIs above.</t>
         </is>

</xml_diff>